<commit_message>
feat: add includeFileSources option for multi-file imports to show file names in first column
</commit_message>
<xml_diff>
--- a/trials/2026-03-06-java-scope-001/exports/java-scope-001.xlsx
+++ b/trials/2026-03-06-java-scope-001/exports/java-scope-001.xlsx
@@ -58,12 +58,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>src</t>
         </is>
       </c>
@@ -71,16 +76,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>FooController.java</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>package com.example;</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FooController.java</t>
+        </is>
+      </c>
+      <c r="B3"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>FooController.java</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>public class FooController {</t>
         </is>
       </c>
@@ -88,6 +108,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>FooController.java</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t xml:space="preserve">    public String foo() {</t>
         </is>
       </c>
@@ -95,6 +120,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>FooController.java</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t xml:space="preserve">        return "foo";</t>
         </is>
       </c>
@@ -102,6 +132,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>FooController.java</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t xml:space="preserve">    }</t>
         </is>
       </c>
@@ -109,6 +144,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>FooController.java</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>}</t>
         </is>
       </c>
@@ -116,16 +156,31 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>BarService.java</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>package com.example;</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BarService.java</t>
+        </is>
+      </c>
+      <c r="B10"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>BarService.java</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>public class BarService {</t>
         </is>
       </c>
@@ -133,6 +188,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>BarService.java</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t xml:space="preserve">    public void bar() {</t>
         </is>
       </c>
@@ -140,6 +200,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>BarService.java</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t xml:space="preserve">        System.out.println("bar");</t>
         </is>
       </c>
@@ -147,12 +212,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>BarService.java</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t xml:space="preserve">    }</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
+        <is>
+          <t>BarService.java</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>}</t>
         </is>

</xml_diff>